<commit_message>
AP-06: Daten Jahrgang 5 uebertragen
Jg5.xlsx vollstaendig gefuellt: 23 Slots, Sonderwochen, 23 Bausteine mit
Gelingensnachweisen, 48 Stationen, 3 Inputs, 5 Coachings (Mo-Fr), 12 Termine
(davon 3 Entfall), 1 Rasterzeitraum. Quelle: anhang/slots_2026-27.json,
bausteinzeitraum-uebersicht.jpg und SOUL Artefakt Klasse 5 (siehe
Bericht). tools/fill_jg5.mjs ist das wiederholbare Erzeugungsskript dazu.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg5.xlsx
+++ b/content/jahrgaenge/Jg5.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="312">
   <si>
     <t>Hinweise zu Jg5.xlsx</t>
   </si>
@@ -497,14 +497,474 @@
   </si>
   <si>
     <t>Bausteinzeitraum 31.08. bis 02.10.2026</t>
+  </si>
+  <si>
+    <t>Kennenlernwoche</t>
+  </si>
+  <si>
+    <t>kennenlernen</t>
+  </si>
+  <si>
+    <t>SOUL-Einführungswoche + SOUL-Basics 1</t>
+  </si>
+  <si>
+    <t>einfuehrung</t>
+  </si>
+  <si>
+    <t>SOUL-Basics Woche</t>
+  </si>
+  <si>
+    <t>soul-basics</t>
+  </si>
+  <si>
+    <t>Pufferwoche + SOUL Basics + Weihnachtsmarkt</t>
+  </si>
+  <si>
+    <t>puffer</t>
+  </si>
+  <si>
+    <t>Besinn-Dich-Tage</t>
+  </si>
+  <si>
+    <t>besinntage</t>
+  </si>
+  <si>
+    <t>letzte Schulwoche</t>
+  </si>
+  <si>
+    <t>letzte-woche</t>
+  </si>
+  <si>
+    <t>jg5-ma-1</t>
+  </si>
+  <si>
+    <t>ma</t>
+  </si>
+  <si>
+    <t>jg5-de-2</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>jg5-en-1</t>
+  </si>
+  <si>
+    <t>en</t>
+  </si>
+  <si>
+    <t>jg5-geo-1</t>
+  </si>
+  <si>
+    <t>geo</t>
+  </si>
+  <si>
+    <t>jg5-de-3</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>jg5-ma-2</t>
+  </si>
+  <si>
+    <t>jg5-bio-2</t>
+  </si>
+  <si>
+    <t>jg5-de-5</t>
+  </si>
+  <si>
+    <t>jg5-en-2</t>
+  </si>
+  <si>
+    <t>jg5-geo-2</t>
+  </si>
+  <si>
+    <t>jg5-de-4</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>jg5-ma-3</t>
+  </si>
+  <si>
+    <t>jg5-bio-3</t>
+  </si>
+  <si>
+    <t>jg5-de-6</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>jg5-en-3</t>
+  </si>
+  <si>
+    <t>jg5-geo-3</t>
+  </si>
+  <si>
+    <t>jg5-ma-4</t>
+  </si>
+  <si>
+    <t>jg5-bio-4</t>
+  </si>
+  <si>
+    <t>jg5-de-7</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>jg5-en-4</t>
+  </si>
+  <si>
+    <t>jg5-geo-4</t>
+  </si>
+  <si>
+    <t>Briefe &amp; E-Mails</t>
+  </si>
+  <si>
+    <t>Einen Brief schreiben</t>
+  </si>
+  <si>
+    <t>Grundlagen: Wiederholung</t>
+  </si>
+  <si>
+    <t>Kurzkontrolle</t>
+  </si>
+  <si>
+    <t>Rechtschreibung</t>
+  </si>
+  <si>
+    <t>Grundlagen</t>
+  </si>
+  <si>
+    <t>Die Erde</t>
+  </si>
+  <si>
+    <t>Zeichensetzung</t>
+  </si>
+  <si>
+    <t>Arbeiten mit natürlichen Zahlen</t>
+  </si>
+  <si>
+    <t>Lurche und Reptilien</t>
+  </si>
+  <si>
+    <t>Märchen und Fantasie</t>
+  </si>
+  <si>
+    <t>Welcome to my world</t>
+  </si>
+  <si>
+    <t>Atlasführerschein</t>
+  </si>
+  <si>
+    <t>Wörterbuch</t>
+  </si>
+  <si>
+    <t>geometrische Muster und Formen</t>
+  </si>
+  <si>
+    <t>Vögel</t>
+  </si>
+  <si>
+    <t>Rico, Oskar und die Tieferschatten</t>
+  </si>
+  <si>
+    <t>Holidays</t>
+  </si>
+  <si>
+    <t>Deutschland: Topografie und Küsten</t>
+  </si>
+  <si>
+    <t>Flächeninhalte und Formen</t>
+  </si>
+  <si>
+    <t>Säugetiere</t>
+  </si>
+  <si>
+    <t>Lyrik</t>
+  </si>
+  <si>
+    <t>Party Star</t>
+  </si>
+  <si>
+    <t>Norddeutsches Tiefland und Mittelgebirge</t>
+  </si>
+  <si>
+    <t>Der persönliche Brief: Redemittel</t>
+  </si>
+  <si>
+    <t>M1, A3 oder M2</t>
+  </si>
+  <si>
+    <t>Der persönliche Brief: Übungen</t>
+  </si>
+  <si>
+    <t>wahl</t>
+  </si>
+  <si>
+    <t>M3, M4</t>
+  </si>
+  <si>
+    <t>Der persönliche Brief: Schreibübungen</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>Die Adresse: Aufbau</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Der förmliche Brief: Aufbau</t>
+  </si>
+  <si>
+    <t>A5, A6</t>
+  </si>
+  <si>
+    <t>Der förmliche Brief: Die Höflichkeitsform</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>Der förmliche Brief: Redemittel</t>
+  </si>
+  <si>
+    <t>M5, A7 oder M6</t>
+  </si>
+  <si>
+    <t>Der förmliche Brief: Übungen</t>
+  </si>
+  <si>
+    <t>M7, M8</t>
+  </si>
+  <si>
+    <t>Der förmliche Brief: Schreibübungen</t>
+  </si>
+  <si>
+    <t>A8</t>
+  </si>
+  <si>
+    <t>Der Briefumschlag: Aufbau</t>
+  </si>
+  <si>
+    <t>A9</t>
+  </si>
+  <si>
+    <t>Die Geschichte der Post: Textverständnis</t>
+  </si>
+  <si>
+    <t>M9, A10 oder A11</t>
+  </si>
+  <si>
+    <t>Übungen</t>
+  </si>
+  <si>
+    <t>A12, M10–M14</t>
+  </si>
+  <si>
+    <t>Vergleich Briefe und E-Mails</t>
+  </si>
+  <si>
+    <t>E-Mails schreiben</t>
+  </si>
+  <si>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>Abschluss und Leistungsmessung</t>
+  </si>
+  <si>
+    <t>Diagnose-Parcours</t>
+  </si>
+  <si>
+    <t>Riesenzahlen-Galerie</t>
+  </si>
+  <si>
+    <t>Stellenwerttafel</t>
+  </si>
+  <si>
+    <t>Zahlenstrahl</t>
+  </si>
+  <si>
+    <t>Heft, Laptop</t>
+  </si>
+  <si>
+    <t>Schätzen &amp; Runden</t>
+  </si>
+  <si>
+    <t>Vergleichen &amp; Ordnen</t>
+  </si>
+  <si>
+    <t>Kopfrechen-Werkstatt</t>
+  </si>
+  <si>
+    <t>Schriftlich Rechnen</t>
+  </si>
+  <si>
+    <t>Geschickt Rechnen</t>
+  </si>
+  <si>
+    <t>Division mit Rest</t>
+  </si>
+  <si>
+    <t>Teiler &amp; Teilbarkeit</t>
+  </si>
+  <si>
+    <t>Sachaufgaben-Werkstatt</t>
+  </si>
+  <si>
+    <t>Schätz-Olympiade</t>
+  </si>
+  <si>
+    <t>Welche Zahl bin ich?</t>
+  </si>
+  <si>
+    <t>Magische Quadrate</t>
+  </si>
+  <si>
+    <t>Zweite Aufgaben-Karte</t>
+  </si>
+  <si>
+    <t>Rechengesetze entdecken</t>
+  </si>
+  <si>
+    <t>Primzahlen &amp; Teilbarkeit</t>
+  </si>
+  <si>
+    <t>Arbeitsweisen in der Biologie</t>
+  </si>
+  <si>
+    <t>Lehrbuch</t>
+  </si>
+  <si>
+    <t>Kennzeichen des Lebendigen</t>
+  </si>
+  <si>
+    <t>M1, A1, Lehrbuch</t>
+  </si>
+  <si>
+    <t>Die Vielfalt der Fische</t>
+  </si>
+  <si>
+    <t>A2, A3, Lehrbuch</t>
+  </si>
+  <si>
+    <t>Fisch-Domino</t>
+  </si>
+  <si>
+    <t>M2, Lehrbuch, Fisch-Buch</t>
+  </si>
+  <si>
+    <t>Äußerer und innerer Bau der Fische</t>
+  </si>
+  <si>
+    <t>A4, Lehrbuch</t>
+  </si>
+  <si>
+    <t>Körperform der Fische</t>
+  </si>
+  <si>
+    <t>Experiment, Lehrbuch, M3</t>
+  </si>
+  <si>
+    <t>Haut der Fische</t>
+  </si>
+  <si>
+    <t>M4, Lupe, Fischschuppe</t>
+  </si>
+  <si>
+    <t>Atmung der Fische</t>
+  </si>
+  <si>
+    <t>A5, A6, Lehrbuch, Laptop</t>
+  </si>
+  <si>
+    <t>A4 (ausgefüllt)</t>
+  </si>
+  <si>
+    <t>Teilnahmepflicht, klassenweiser Termin</t>
+  </si>
+  <si>
+    <t>Fortpflanzung und Entwicklung</t>
+  </si>
+  <si>
+    <t>A7, Lehrbuch, Laptop</t>
+  </si>
+  <si>
+    <t>Verhaltensweisen bei Fortpflanzung/Entwicklung</t>
+  </si>
+  <si>
+    <t>M6, M7, A8, Laptop</t>
+  </si>
+  <si>
+    <t>Ernährung der Fische</t>
+  </si>
+  <si>
+    <t>A9, Lehrbuch, Laptop</t>
+  </si>
+  <si>
+    <t>M8, M9, A10</t>
+  </si>
+  <si>
+    <t>Online-Übungen Sofatutor</t>
+  </si>
+  <si>
+    <t>Laptop, Zugangscode</t>
+  </si>
+  <si>
+    <t>jg5-de-persoenlicher-brief</t>
+  </si>
+  <si>
+    <t>Persönlicher Brief</t>
+  </si>
+  <si>
+    <t>jg5-de-foermlicher-brief</t>
+  </si>
+  <si>
+    <t>Förmlicher Brief</t>
+  </si>
+  <si>
+    <t>HEC</t>
+  </si>
+  <si>
+    <t>RIK</t>
+  </si>
+  <si>
+    <t>HER</t>
+  </si>
+  <si>
+    <t>TRY</t>
+  </si>
+  <si>
+    <t>Kommt mit euren Fragen!</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>entfall</t>
+  </si>
+  <si>
+    <t>Kein Coaching</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -553,7 +1013,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1925,13 +2385,13 @@
     <mergeCell ref="B72:D72"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1953,10 +2413,24 @@
         <v>31</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" s="5">
+        <v>46265</v>
+      </c>
+      <c r="C2" s="5">
+        <v>46297</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1992,27 +2466,35 @@
       <c r="A2">
         <v>5</v>
       </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
       <c r="C2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="5"/>
+      <c r="D2" s="5">
+        <v>46321</v>
+      </c>
       <c r="E2" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"verspielt,klar,sachlich"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"verspielt,klar,sachlich"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="13" style="5" customWidth="1"/>
@@ -2034,21 +2516,122 @@
         <v>34</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
+        <v>46251</v>
+      </c>
+      <c r="B2" s="5">
+        <v>46255</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
+        <v>46258</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46262</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>46279</v>
+      </c>
+      <c r="B4" s="5">
+        <v>46283</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>46300</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46304</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>46370</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46374</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>46468</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46472</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>46573</v>
+      </c>
+      <c r="B8" s="5">
+        <v>46577</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" t="s">
+        <v>170</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="D10:D500">
+      <formula1>"themenwoche,soul-basics,puffer,kennenlernen,einfuehrung,besinntage,fvu,letzte-woche,sonstiges"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:D500">
       <formula1>"themenwoche,soul-basics,puffer,kennenlernen,einfuehrung,besinntage,fvu,letzte-woche,sonstiges"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2099,24 +2682,904 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5">
+        <v>8</v>
+      </c>
+      <c r="G2" s="5">
+        <v>46265</v>
+      </c>
+      <c r="H2" s="5">
+        <v>46297</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" t="s">
+        <v>41</v>
+      </c>
+      <c r="K2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="5">
+        <v>16</v>
+      </c>
+      <c r="G3" s="5">
+        <v>46265</v>
+      </c>
+      <c r="H3" s="5">
+        <v>46297</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J3" t="s">
+        <v>171</v>
+      </c>
+      <c r="K3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="5">
+        <v>16</v>
+      </c>
+      <c r="G4" s="5">
+        <v>46265</v>
+      </c>
+      <c r="H4" s="5">
+        <v>46297</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" t="s">
+        <v>70</v>
+      </c>
+      <c r="K4" t="s">
+        <v>65</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="5">
+        <v>16</v>
+      </c>
+      <c r="G5" s="5">
+        <v>46321</v>
+      </c>
+      <c r="H5" s="5">
+        <v>46346</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" t="s">
+        <v>173</v>
+      </c>
+      <c r="K5" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5">
+        <v>8</v>
+      </c>
+      <c r="G6" s="5">
+        <v>46321</v>
+      </c>
+      <c r="H6" s="5">
+        <v>46346</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" t="s">
+        <v>175</v>
+      </c>
+      <c r="K6" t="s">
+        <v>65</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="5">
+        <v>16</v>
+      </c>
+      <c r="G7" s="5">
+        <v>46321</v>
+      </c>
+      <c r="H7" s="5">
+        <v>46346</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" t="s">
+        <v>177</v>
+      </c>
+      <c r="K7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="5">
+        <v>8</v>
+      </c>
+      <c r="G8" s="5">
+        <v>46349</v>
+      </c>
+      <c r="H8" s="5">
+        <v>46395</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J8" t="s">
+        <v>179</v>
+      </c>
+      <c r="K8" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" t="s">
+        <v>172</v>
+      </c>
+      <c r="C9" t="s">
+        <v>174</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="5">
+        <v>16</v>
+      </c>
+      <c r="G9" s="5">
+        <v>46349</v>
+      </c>
+      <c r="H9" s="5">
+        <v>46395</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J9" t="s">
+        <v>181</v>
+      </c>
+      <c r="K9" t="s">
+        <v>65</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" t="s">
+        <v>174</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="5">
+        <v>16</v>
+      </c>
+      <c r="G10" s="5">
+        <v>46349</v>
+      </c>
+      <c r="H10" s="5">
+        <v>46395</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J10" t="s">
+        <v>182</v>
+      </c>
+      <c r="K10" t="s">
+        <v>65</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="5">
+        <v>16</v>
+      </c>
+      <c r="G11" s="5">
+        <v>46398</v>
+      </c>
+      <c r="H11" s="5">
+        <v>46423</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J11" t="s">
+        <v>183</v>
+      </c>
+      <c r="K11" t="s">
+        <v>65</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>184</v>
+      </c>
+      <c r="B12" t="s">
+        <v>176</v>
+      </c>
+      <c r="C12" t="s">
+        <v>174</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="5">
+        <v>8</v>
+      </c>
+      <c r="G12" s="5">
+        <v>46398</v>
+      </c>
+      <c r="H12" s="5">
+        <v>46423</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J12" t="s">
+        <v>184</v>
+      </c>
+      <c r="K12" t="s">
+        <v>65</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>185</v>
+      </c>
+      <c r="B13" t="s">
+        <v>178</v>
+      </c>
+      <c r="C13" t="s">
+        <v>174</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="5">
+        <v>16</v>
+      </c>
+      <c r="G13" s="5">
+        <v>46398</v>
+      </c>
+      <c r="H13" s="5">
+        <v>46423</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J13" t="s">
+        <v>185</v>
+      </c>
+      <c r="K13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>187</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="5">
+        <v>8</v>
+      </c>
+      <c r="G14" s="5">
+        <v>46440</v>
+      </c>
+      <c r="H14" s="5">
+        <v>46465</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J14" t="s">
+        <v>186</v>
+      </c>
+      <c r="K14" t="s">
+        <v>65</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" t="s">
+        <v>172</v>
+      </c>
+      <c r="C15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="5">
+        <v>16</v>
+      </c>
+      <c r="G15" s="5">
+        <v>46440</v>
+      </c>
+      <c r="H15" s="5">
+        <v>46465</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J15" t="s">
+        <v>188</v>
+      </c>
+      <c r="K15" t="s">
+        <v>65</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" t="s">
+        <v>180</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="5">
+        <v>16</v>
+      </c>
+      <c r="G16" s="5">
+        <v>46440</v>
+      </c>
+      <c r="H16" s="5">
+        <v>46465</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J16" t="s">
+        <v>189</v>
+      </c>
+      <c r="K16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>191</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="5">
+        <v>24</v>
+      </c>
+      <c r="G17" s="5">
+        <v>46482</v>
+      </c>
+      <c r="H17" s="5">
+        <v>46542</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J17" t="s">
+        <v>190</v>
+      </c>
+      <c r="K17" t="s">
+        <v>65</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>192</v>
+      </c>
+      <c r="B18" t="s">
+        <v>176</v>
+      </c>
+      <c r="C18" t="s">
+        <v>180</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="5">
+        <v>8</v>
+      </c>
+      <c r="G18" s="5">
+        <v>46482</v>
+      </c>
+      <c r="H18" s="5">
+        <v>46507</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J18" t="s">
+        <v>192</v>
+      </c>
+      <c r="K18" t="s">
+        <v>65</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>193</v>
+      </c>
+      <c r="B19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C19" t="s">
+        <v>180</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="5">
+        <v>16</v>
+      </c>
+      <c r="G19" s="5">
+        <v>46482</v>
+      </c>
+      <c r="H19" s="5">
+        <v>46507</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" t="s">
+        <v>193</v>
+      </c>
+      <c r="K19" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B20" t="s">
+        <v>172</v>
+      </c>
+      <c r="C20" t="s">
+        <v>187</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="5">
+        <v>16</v>
+      </c>
+      <c r="G20" s="5">
+        <v>46510</v>
+      </c>
+      <c r="H20" s="5">
+        <v>46542</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J20" t="s">
+        <v>194</v>
+      </c>
+      <c r="K20" t="s">
+        <v>65</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>195</v>
+      </c>
+      <c r="B21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" t="s">
+        <v>187</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="5">
+        <v>16</v>
+      </c>
+      <c r="G21" s="5">
+        <v>46510</v>
+      </c>
+      <c r="H21" s="5">
+        <v>46542</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J21" t="s">
+        <v>195</v>
+      </c>
+      <c r="K21" t="s">
+        <v>65</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" t="s">
+        <v>197</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="5">
+        <v>16</v>
+      </c>
+      <c r="G22" s="5">
+        <v>46545</v>
+      </c>
+      <c r="H22" s="5">
+        <v>46570</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J22" t="s">
+        <v>196</v>
+      </c>
+      <c r="K22" t="s">
+        <v>65</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B23" t="s">
+        <v>176</v>
+      </c>
+      <c r="C23" t="s">
+        <v>187</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="5">
+        <v>8</v>
+      </c>
+      <c r="G23" s="5">
+        <v>46545</v>
+      </c>
+      <c r="H23" s="5">
+        <v>46570</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J23" t="s">
+        <v>198</v>
+      </c>
+      <c r="K23" t="s">
+        <v>65</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>199</v>
+      </c>
+      <c r="B24" t="s">
+        <v>178</v>
+      </c>
+      <c r="C24" t="s">
+        <v>187</v>
+      </c>
+      <c r="D24">
+        <v>3</v>
+      </c>
+      <c r="E24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="5">
+        <v>16</v>
+      </c>
+      <c r="G24" s="5">
+        <v>46545</v>
+      </c>
+      <c r="H24" s="5">
+        <v>46570</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J24" t="s">
+        <v>199</v>
+      </c>
+      <c r="K24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="K10:K500">
+      <formula1>"fest,wahl,vorlaeufig,offen"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="K2:K500">
       <formula1>"fest,wahl,vorlaeufig,offen"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2155,21 +3618,496 @@
         <v>85</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" t="s">
+        <v>172</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>184</v>
+      </c>
+      <c r="B12" t="s">
+        <v>176</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>185</v>
+      </c>
+      <c r="B13" t="s">
+        <v>178</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" t="s">
+        <v>172</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>192</v>
+      </c>
+      <c r="B18" t="s">
+        <v>176</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>193</v>
+      </c>
+      <c r="B19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B20" t="s">
+        <v>172</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>195</v>
+      </c>
+      <c r="B21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B23" t="s">
+        <v>176</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>199</v>
+      </c>
+      <c r="B24" t="s">
+        <v>178</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2206,21 +4144,1272 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D4" t="s">
+        <v>227</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" t="s">
+        <v>93</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E9">
+        <v>30</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D10" t="s">
+        <v>227</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="D12" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12">
+        <v>20</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D13" t="s">
+        <v>227</v>
+      </c>
+      <c r="E13">
+        <v>30</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D14" t="s">
+        <v>227</v>
+      </c>
+      <c r="E14">
+        <v>60</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D15" t="s">
+        <v>227</v>
+      </c>
+      <c r="E15">
+        <v>20</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D16" t="s">
+        <v>227</v>
+      </c>
+      <c r="E16">
+        <v>20</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17">
+        <v>30</v>
+      </c>
+      <c r="F17">
+        <v>3</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D18" t="s">
+        <v>93</v>
+      </c>
+      <c r="E18">
+        <v>45</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>171</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D19" t="s">
+        <v>93</v>
+      </c>
+      <c r="E19">
+        <v>45</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>171</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D20" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20">
+        <v>45</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>171</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D21" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21">
+        <v>45</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>171</v>
+      </c>
+      <c r="B22">
+        <v>5</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="D22" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22">
+        <v>45</v>
+      </c>
+      <c r="F22">
+        <v>2</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>171</v>
+      </c>
+      <c r="B23">
+        <v>6</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23">
+        <v>45</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>171</v>
+      </c>
+      <c r="B24">
+        <v>7</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="D24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24">
+        <v>45</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>171</v>
+      </c>
+      <c r="B25">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D25" t="s">
+        <v>93</v>
+      </c>
+      <c r="E25">
+        <v>45</v>
+      </c>
+      <c r="F25">
+        <v>2</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>171</v>
+      </c>
+      <c r="B26">
+        <v>9</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="D26" t="s">
+        <v>93</v>
+      </c>
+      <c r="E26">
+        <v>45</v>
+      </c>
+      <c r="F26">
+        <v>2</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27">
+        <v>10</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D27" t="s">
+        <v>93</v>
+      </c>
+      <c r="E27">
+        <v>45</v>
+      </c>
+      <c r="F27">
+        <v>2</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28">
+        <v>11</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="D28" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28">
+        <v>45</v>
+      </c>
+      <c r="F28">
+        <v>2</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29">
+        <v>12</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="D29" t="s">
+        <v>93</v>
+      </c>
+      <c r="E29">
+        <v>45</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>171</v>
+      </c>
+      <c r="B30">
+        <v>13</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D30" t="s">
+        <v>227</v>
+      </c>
+      <c r="E30">
+        <v>30</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>171</v>
+      </c>
+      <c r="B31">
+        <v>14</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D31" t="s">
+        <v>227</v>
+      </c>
+      <c r="E31">
+        <v>30</v>
+      </c>
+      <c r="F31">
+        <v>3</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>171</v>
+      </c>
+      <c r="B32">
+        <v>15</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="D32" t="s">
+        <v>227</v>
+      </c>
+      <c r="E32">
+        <v>30</v>
+      </c>
+      <c r="F32">
+        <v>2</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>171</v>
+      </c>
+      <c r="B33">
+        <v>16</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D33" t="s">
+        <v>227</v>
+      </c>
+      <c r="E33">
+        <v>30</v>
+      </c>
+      <c r="F33">
+        <v>2</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>171</v>
+      </c>
+      <c r="B34">
+        <v>17</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D34" t="s">
+        <v>227</v>
+      </c>
+      <c r="E34">
+        <v>30</v>
+      </c>
+      <c r="F34">
+        <v>3</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>171</v>
+      </c>
+      <c r="B35">
+        <v>18</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D35" t="s">
+        <v>227</v>
+      </c>
+      <c r="E35">
+        <v>30</v>
+      </c>
+      <c r="F35">
+        <v>3</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D36" t="s">
+        <v>93</v>
+      </c>
+      <c r="E36">
+        <v>30</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>70</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D37" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37">
+        <v>60</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38">
+        <v>3</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D38" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38">
+        <v>90</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39">
+        <v>4</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D39" t="s">
+        <v>227</v>
+      </c>
+      <c r="E39">
+        <v>30</v>
+      </c>
+      <c r="F39">
+        <v>3</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40">
+        <v>5</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="D40" t="s">
+        <v>93</v>
+      </c>
+      <c r="E40">
+        <v>45</v>
+      </c>
+      <c r="F40">
+        <v>2</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>70</v>
+      </c>
+      <c r="B41">
+        <v>6</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D41" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41">
+        <v>45</v>
+      </c>
+      <c r="F41">
+        <v>2</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42">
+        <v>7</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D42" t="s">
+        <v>93</v>
+      </c>
+      <c r="E42">
+        <v>30</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>70</v>
+      </c>
+      <c r="B43">
+        <v>8</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D43" t="s">
+        <v>93</v>
+      </c>
+      <c r="E43">
+        <v>45</v>
+      </c>
+      <c r="F43">
+        <v>2</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44">
+        <v>9</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" t="s">
+        <v>93</v>
+      </c>
+      <c r="E44">
+        <v>30</v>
+      </c>
+      <c r="F44">
+        <v>2</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45">
+        <v>10</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D45" t="s">
+        <v>93</v>
+      </c>
+      <c r="E45">
+        <v>45</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>70</v>
+      </c>
+      <c r="B46">
+        <v>11</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D46" t="s">
+        <v>227</v>
+      </c>
+      <c r="E46">
+        <v>30</v>
+      </c>
+      <c r="F46">
+        <v>2</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>70</v>
+      </c>
+      <c r="B47">
+        <v>12</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D47" t="s">
+        <v>93</v>
+      </c>
+      <c r="E47">
+        <v>60</v>
+      </c>
+      <c r="F47">
+        <v>3</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>70</v>
+      </c>
+      <c r="B48">
+        <v>13</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D48" t="s">
+        <v>93</v>
+      </c>
+      <c r="E48">
+        <v>120</v>
+      </c>
+      <c r="F48">
+        <v>3</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>70</v>
+      </c>
+      <c r="B49">
+        <v>14</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D49" t="s">
+        <v>227</v>
+      </c>
+      <c r="E49">
+        <v>60</v>
+      </c>
+      <c r="F49">
+        <v>2</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="D10:D500">
+      <formula1>"pflicht,wahl"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:D500">
       <formula1>"pflicht,wahl"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -2253,27 +5442,105 @@
         <v>115</v>
       </c>
     </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>301</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
-  <dataValidations count="3">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="C10:C500">
+      <formula1>"fach,methode,baustein"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C2:C500">
       <formula1>"fach,methode,baustein"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F10:F500">
+      <formula1>"ja,nein"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F2:F500">
       <formula1>"ja,nein"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2298,24 +5565,115 @@
         <v>130</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C2" s="5">
+        <v>46272</v>
+      </c>
+      <c r="D2" s="5">
+        <v>46297</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C3" s="5">
+        <v>46272</v>
+      </c>
+      <c r="D3" s="5">
+        <v>46297</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>304</v>
+      </c>
+      <c r="C4" s="5">
+        <v>46272</v>
+      </c>
+      <c r="D4" s="5">
+        <v>46297</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>305</v>
+      </c>
+      <c r="C5" s="5">
+        <v>46272</v>
+      </c>
+      <c r="D5" s="5">
+        <v>46297</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="5">
+        <v>46272</v>
+      </c>
+      <c r="D6" s="5">
+        <v>46297</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" sqref="A10:A500">
+      <formula1>"Mo,Di,Mi,Do,Fr"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="A2:A500">
       <formula1>"Mo,Di,Mi,Do,Fr"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="E10:E500">
+      <formula1>"A,B,C"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E2:E500">
       <formula1>"A,B,C"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" style="5" customWidth="1"/>
@@ -2359,23 +5717,419 @@
         <v>149</v>
       </c>
     </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
+        <v>46273</v>
+      </c>
+      <c r="B2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2">
+        <v>9</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
+        <v>46274</v>
+      </c>
+      <c r="B3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>306</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" t="s">
+        <v>299</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>46276</v>
+      </c>
+      <c r="B4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" t="s">
+        <v>172</v>
+      </c>
+      <c r="D4" t="s">
+        <v>303</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>46287</v>
+      </c>
+      <c r="B5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E5" t="s">
+        <v>308</v>
+      </c>
+      <c r="F5" t="s">
+        <v>106</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5">
+        <v>9</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>46288</v>
+      </c>
+      <c r="B6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" t="s">
+        <v>306</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>301</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>46290</v>
+      </c>
+      <c r="B7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C7" t="s">
+        <v>172</v>
+      </c>
+      <c r="D7" t="s">
+        <v>303</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H7" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>46294</v>
+      </c>
+      <c r="B8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E8" t="s">
+        <v>309</v>
+      </c>
+      <c r="F8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8">
+        <v>9</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>46295</v>
+      </c>
+      <c r="B9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
+        <v>306</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H9" t="s">
+        <v>8</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>46297</v>
+      </c>
+      <c r="B10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C10" t="s">
+        <v>172</v>
+      </c>
+      <c r="D10" t="s">
+        <v>303</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H10" t="s">
+        <v>8</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>46287</v>
+      </c>
+      <c r="B11" t="s">
+        <v>310</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>303</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H11" t="s">
+        <v>8</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>46296</v>
+      </c>
+      <c r="B12" t="s">
+        <v>310</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>305</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H12" t="s">
+        <v>8</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>46297</v>
+      </c>
+      <c r="B13" t="s">
+        <v>310</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>140</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>8</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
-  <dataValidations count="4">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" sqref="B10:B500">
+      <formula1>"input,coaching,sonstiges,entfall"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="B2:B500">
       <formula1>"input,coaching,sonstiges,entfall"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="C10:C500">
+      <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C2:C500">
       <formula1>"de,ma,en,bio,geo,fvu,offen"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="E10:E500">
+      <formula1>"A,B,C"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E2:E500">
       <formula1>"A,B,C"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I10:I500">
+      <formula1>"ja,nein"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="I2:I500">
       <formula1>"ja,nein"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Wochenraster: alle Bausteinzeitraeume fuer Jg5, Jg6 und Jg7 angelegt
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg5.xlsx
+++ b/content/jahrgaenge/Jg5.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3107" uniqueCount="839">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="861">
   <si>
     <t>Hinweise zu Jg5.xlsx</t>
   </si>
@@ -2537,6 +2537,72 @@
   </si>
   <si>
     <t>2027-07-01</t>
+  </si>
+  <si>
+    <t>jg5-r2</t>
+  </si>
+  <si>
+    <t>Bausteinzeitraum 26.10. bis 20.11.2026</t>
+  </si>
+  <si>
+    <t>jg5-r3</t>
+  </si>
+  <si>
+    <t>Bausteinzeitraum 23.11. bis 08.01.2027</t>
+  </si>
+  <si>
+    <t>jg5-r4</t>
+  </si>
+  <si>
+    <t>2027-01-11</t>
+  </si>
+  <si>
+    <t>2027-02-05</t>
+  </si>
+  <si>
+    <t>Bausteinzeitraum 11.01. bis 05.02.2027</t>
+  </si>
+  <si>
+    <t>jg5-r5</t>
+  </si>
+  <si>
+    <t>2027-02-22</t>
+  </si>
+  <si>
+    <t>Bausteinzeitraum 22.02. bis 19.03.2027</t>
+  </si>
+  <si>
+    <t>jg5-r6</t>
+  </si>
+  <si>
+    <t>2027-04-05</t>
+  </si>
+  <si>
+    <t>Bausteinzeitraum 05.04. bis 30.04.2027</t>
+  </si>
+  <si>
+    <t>jg5-r7</t>
+  </si>
+  <si>
+    <t>2027-05-03</t>
+  </si>
+  <si>
+    <t>2027-06-04</t>
+  </si>
+  <si>
+    <t>Bausteinzeitraum 03.05. bis 04.06.2027</t>
+  </si>
+  <si>
+    <t>jg5-r8</t>
+  </si>
+  <si>
+    <t>2027-06-07</t>
+  </si>
+  <si>
+    <t>2027-07-02</t>
+  </si>
+  <si>
+    <t>Bausteinzeitraum 07.06. bis 02.07.2027</t>
   </si>
 </sst>
 </file>
@@ -3972,7 +4038,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -4006,6 +4072,104 @@
       </c>
       <c r="D2" s="2" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>839</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>734</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>841</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>735</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>757</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>843</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>844</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>845</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>847</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>848</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>792</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>850</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>851</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>810</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>853</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>857</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>858</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>859</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>860</v>
       </c>
     </row>
   </sheetData>

</xml_diff>